<commit_message>
Add NA49 1999 2011
</commit_message>
<xml_diff>
--- a/BT/experimentData/raw/NA49 158AGeV.xlsx
+++ b/BT/experimentData/raw/NA49 158AGeV.xlsx
@@ -5,15 +5,16 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-20.04\home\xiaozhou\WorkSpace\NuclearModel\tglaubermc\runglauber_v3.3\BT\expData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu-20.04\home\xiaozhou\WorkSpace\NuclearModel\tglaubermc\runglauber_v3.3\BT\experimentData\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B823EB4-F99E-490B-84B9-F817D0F80B2F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AD84A72-C084-4D18-B248-0165431E3B51}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="30720" windowHeight="13332" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="30720" windowHeight="13332" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="2011 158A" sheetId="1" r:id="rId1"/>
+    <sheet name="1999 158A" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="12">
   <si>
     <t>y区间</t>
   </si>
@@ -45,14 +46,6 @@
     <t>dn/dy</t>
   </si>
   <si>
-    <t>ylow</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>yup</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>dN/dy</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -63,6 +56,17 @@
   <si>
     <t>https://link.aps.org/doi/10.1103/PhysRevC.83.014901</t>
     <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>dylow</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>dyup</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t># Format: x y -dx +dx -dy +dy</t>
   </si>
 </sst>
 </file>
@@ -405,7 +409,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AA18"/>
+  <dimension ref="A1:AA27"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="13" max="19" width="0" hidden="1" customWidth="1"/>
@@ -413,19 +417,19 @@
   <sheetData>
     <row r="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="X1" t="s">
+        <v>9</v>
+      </c>
+      <c r="Y1" t="s">
         <v>10</v>
       </c>
-      <c r="X1" t="s">
+      <c r="Z1" t="s">
         <v>6</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="AA1" t="s">
         <v>7</v>
-      </c>
-      <c r="Z1" t="s">
-        <v>8</v>
-      </c>
-      <c r="AA1" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:27" ht="15" x14ac:dyDescent="0.35">
@@ -501,11 +505,11 @@
         <v>-3.23</v>
       </c>
       <c r="Z2">
-        <f>I2-T2</f>
+        <f t="shared" ref="Z2:Z12" si="0">I2-T2</f>
         <v>24.02</v>
       </c>
       <c r="AA2">
-        <f>2*Z2/352</f>
+        <f t="shared" ref="AA2:AA12" si="1">2*Z2/352</f>
         <v>0.13647727272727272</v>
       </c>
     </row>
@@ -553,19 +557,19 @@
         <v>0.13</v>
       </c>
       <c r="X3">
-        <f t="shared" ref="X3:X12" si="0">B3-2.91</f>
+        <f t="shared" ref="X3:X12" si="2">B3-2.91</f>
         <v>-3.23</v>
       </c>
       <c r="Y3">
-        <f t="shared" ref="Y3:Y12" si="1">F3-2.91</f>
+        <f t="shared" ref="Y3:Y12" si="3">F3-2.91</f>
         <v>-3.0300000000000002</v>
       </c>
       <c r="Z3">
-        <f>I3-T3</f>
+        <f t="shared" si="0"/>
         <v>25.88</v>
       </c>
       <c r="AA3">
-        <f>2*Z3/352</f>
+        <f t="shared" si="1"/>
         <v>0.14704545454545453</v>
       </c>
     </row>
@@ -634,19 +638,19 @@
         <v>0.12</v>
       </c>
       <c r="X4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>-3.0300000000000002</v>
       </c>
       <c r="Y4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>-2.83</v>
       </c>
       <c r="Z4">
-        <f>I4-T4</f>
+        <f t="shared" si="0"/>
         <v>25.76</v>
       </c>
       <c r="AA4">
-        <f>2*Z4/352</f>
+        <f t="shared" si="1"/>
         <v>0.14636363636363636</v>
       </c>
     </row>
@@ -694,19 +698,19 @@
         <v>0.12</v>
       </c>
       <c r="X5">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>-2.83</v>
       </c>
       <c r="Y5">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>-2.63</v>
       </c>
       <c r="Z5">
-        <f>I5-T5</f>
+        <f t="shared" si="0"/>
         <v>26.32</v>
       </c>
       <c r="AA5">
-        <f>2*Z5/352</f>
+        <f t="shared" si="1"/>
         <v>0.14954545454545454</v>
       </c>
     </row>
@@ -775,19 +779,19 @@
         <v>0.11</v>
       </c>
       <c r="X6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>-2.63</v>
       </c>
       <c r="Y6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>-2.4300000000000002</v>
       </c>
       <c r="Z6">
-        <f>I6-T6</f>
+        <f t="shared" si="0"/>
         <v>26.169999999999998</v>
       </c>
       <c r="AA6">
-        <f>2*Z6/352</f>
+        <f t="shared" si="1"/>
         <v>0.14869318181818181</v>
       </c>
     </row>
@@ -835,19 +839,19 @@
         <v>0.11</v>
       </c>
       <c r="X7">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>-2.4300000000000002</v>
       </c>
       <c r="Y7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>-2.23</v>
       </c>
       <c r="Z7">
-        <f>I7-T7</f>
+        <f t="shared" si="0"/>
         <v>27.439999999999998</v>
       </c>
       <c r="AA7">
-        <f>2*Z7/352</f>
+        <f t="shared" si="1"/>
         <v>0.15590909090909089</v>
       </c>
     </row>
@@ -916,19 +920,19 @@
         <v>0.1</v>
       </c>
       <c r="X8">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>-2.23</v>
       </c>
       <c r="Y8">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>-2.0300000000000002</v>
       </c>
       <c r="Z8">
-        <f>I8-T8</f>
+        <f t="shared" si="0"/>
         <v>29.990000000000002</v>
       </c>
       <c r="AA8">
-        <f>2*Z8/352</f>
+        <f t="shared" si="1"/>
         <v>0.17039772727272728</v>
       </c>
     </row>
@@ -976,19 +980,19 @@
         <v>0.1</v>
       </c>
       <c r="X9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>-2.0300000000000002</v>
       </c>
       <c r="Y9">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>-1.83</v>
       </c>
       <c r="Z9">
-        <f>I9-T9</f>
+        <f t="shared" si="0"/>
         <v>29.200000000000003</v>
       </c>
       <c r="AA9">
-        <f>2*Z9/352</f>
+        <f t="shared" si="1"/>
         <v>0.16590909090909092</v>
       </c>
     </row>
@@ -1057,19 +1061,19 @@
         <v>0.1</v>
       </c>
       <c r="X10">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>-1.83</v>
       </c>
       <c r="Y10">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>-1.6300000000000001</v>
       </c>
       <c r="Z10">
-        <f>I10-T10</f>
+        <f t="shared" si="0"/>
         <v>31.75</v>
       </c>
       <c r="AA10">
-        <f>2*Z10/352</f>
+        <f t="shared" si="1"/>
         <v>0.18039772727272727</v>
       </c>
     </row>
@@ -1117,19 +1121,19 @@
         <v>0.1</v>
       </c>
       <c r="X11">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>-1.6300000000000001</v>
       </c>
       <c r="Y11">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>-1.4300000000000002</v>
       </c>
       <c r="Z11">
-        <f>I11-T11</f>
+        <f t="shared" si="0"/>
         <v>38.24</v>
       </c>
       <c r="AA11">
-        <f>2*Z11/352</f>
+        <f t="shared" si="1"/>
         <v>0.21727272727272728</v>
       </c>
     </row>
@@ -1174,19 +1178,19 @@
         <v>0</v>
       </c>
       <c r="X12">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>-1.4300000000000002</v>
       </c>
       <c r="Y12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>-1.2300000000000002</v>
       </c>
       <c r="Z12">
-        <f>I12-T12</f>
+        <f t="shared" si="0"/>
         <v>39.35</v>
       </c>
       <c r="AA12">
-        <f>2*Z12/352</f>
+        <f t="shared" si="1"/>
         <v>0.22357954545454548</v>
       </c>
     </row>
@@ -1199,11 +1203,260 @@
     <row r="16" spans="1:27" ht="15" x14ac:dyDescent="0.35">
       <c r="A16" s="1"/>
     </row>
-    <row r="17" spans="1:1" ht="15" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:9" ht="15" x14ac:dyDescent="0.35">
       <c r="A17" s="1"/>
-    </row>
-    <row r="18" spans="1:1" ht="15" x14ac:dyDescent="0.35">
+      <c r="D17">
+        <f>(E17+F17)/2</f>
+        <v>-0.42000000000000004</v>
+      </c>
+      <c r="E17">
+        <v>-0.52</v>
+      </c>
+      <c r="F17">
+        <v>-0.32</v>
+      </c>
+      <c r="G17">
+        <v>24.02</v>
+      </c>
+      <c r="H17">
+        <f t="shared" ref="H17:H27" si="4">SQRT(K2*K2+V2*V2)</f>
+        <v>1.4159802258506295</v>
+      </c>
+      <c r="I17">
+        <f>G17*0.07</f>
+        <v>1.6814000000000002</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="15" x14ac:dyDescent="0.35">
       <c r="A18" s="1"/>
+      <c r="D18">
+        <f t="shared" ref="D18:D27" si="5">(E18+F18)/2</f>
+        <v>-0.22</v>
+      </c>
+      <c r="E18">
+        <v>-0.32</v>
+      </c>
+      <c r="F18">
+        <v>-0.12</v>
+      </c>
+      <c r="G18">
+        <v>25.88</v>
+      </c>
+      <c r="H18">
+        <f t="shared" si="4"/>
+        <v>1.2467958934805647</v>
+      </c>
+      <c r="I18">
+        <f t="shared" ref="I18:I27" si="6">G18*0.07</f>
+        <v>1.8116000000000001</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="D19">
+        <f t="shared" si="5"/>
+        <v>-1.9999999999999997E-2</v>
+      </c>
+      <c r="E19">
+        <v>-0.12</v>
+      </c>
+      <c r="F19">
+        <v>0.08</v>
+      </c>
+      <c r="G19">
+        <v>25.76</v>
+      </c>
+      <c r="H19">
+        <f t="shared" si="4"/>
+        <v>1.0965856099730655</v>
+      </c>
+      <c r="I19">
+        <f t="shared" si="6"/>
+        <v>1.8032000000000004</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="D20">
+        <f t="shared" si="5"/>
+        <v>0.18000000000000002</v>
+      </c>
+      <c r="E20">
+        <v>0.08</v>
+      </c>
+      <c r="F20">
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="G20">
+        <v>26.32</v>
+      </c>
+      <c r="H20">
+        <f t="shared" si="4"/>
+        <v>1.0171037311896953</v>
+      </c>
+      <c r="I20">
+        <f t="shared" si="6"/>
+        <v>1.8424000000000003</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="D21">
+        <f t="shared" si="5"/>
+        <v>0.38</v>
+      </c>
+      <c r="E21">
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="F21">
+        <v>0.48</v>
+      </c>
+      <c r="G21">
+        <v>26.169999999999998</v>
+      </c>
+      <c r="H21">
+        <f t="shared" si="4"/>
+        <v>0.94641428560646734</v>
+      </c>
+      <c r="I21">
+        <f t="shared" si="6"/>
+        <v>1.8319000000000001</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="D22">
+        <f t="shared" si="5"/>
+        <v>0.58000000000000007</v>
+      </c>
+      <c r="E22">
+        <v>0.48</v>
+      </c>
+      <c r="F22">
+        <v>0.68</v>
+      </c>
+      <c r="G22">
+        <v>27.439999999999998</v>
+      </c>
+      <c r="H22">
+        <f t="shared" si="4"/>
+        <v>0.89677198885781439</v>
+      </c>
+      <c r="I22">
+        <f t="shared" si="6"/>
+        <v>1.9208000000000001</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="D23">
+        <f t="shared" si="5"/>
+        <v>0.78</v>
+      </c>
+      <c r="E23">
+        <v>0.68</v>
+      </c>
+      <c r="F23">
+        <v>0.88</v>
+      </c>
+      <c r="G23">
+        <v>29.990000000000002</v>
+      </c>
+      <c r="H23">
+        <f t="shared" si="4"/>
+        <v>0.88566359301938113</v>
+      </c>
+      <c r="I23">
+        <f t="shared" si="6"/>
+        <v>2.0993000000000004</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="D24">
+        <f t="shared" si="5"/>
+        <v>0.98</v>
+      </c>
+      <c r="E24">
+        <v>0.88</v>
+      </c>
+      <c r="F24">
+        <v>1.08</v>
+      </c>
+      <c r="G24">
+        <v>29.200000000000003</v>
+      </c>
+      <c r="H24">
+        <f t="shared" si="4"/>
+        <v>0.85586213843118442</v>
+      </c>
+      <c r="I24">
+        <f t="shared" si="6"/>
+        <v>2.0440000000000005</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="D25">
+        <f t="shared" si="5"/>
+        <v>1.1800000000000002</v>
+      </c>
+      <c r="E25">
+        <v>1.08</v>
+      </c>
+      <c r="F25">
+        <v>1.28</v>
+      </c>
+      <c r="G25">
+        <v>31.75</v>
+      </c>
+      <c r="H25">
+        <f t="shared" si="4"/>
+        <v>1.0547511554864493</v>
+      </c>
+      <c r="I25">
+        <f t="shared" si="6"/>
+        <v>2.2225000000000001</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="D26">
+        <f t="shared" si="5"/>
+        <v>1.38</v>
+      </c>
+      <c r="E26">
+        <v>1.28</v>
+      </c>
+      <c r="F26">
+        <v>1.48</v>
+      </c>
+      <c r="G26">
+        <v>38.24</v>
+      </c>
+      <c r="H26">
+        <f t="shared" si="4"/>
+        <v>3.4314574163174458</v>
+      </c>
+      <c r="I26">
+        <f t="shared" si="6"/>
+        <v>2.6768000000000005</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="D27">
+        <f t="shared" si="5"/>
+        <v>1.58</v>
+      </c>
+      <c r="E27">
+        <v>1.48</v>
+      </c>
+      <c r="F27">
+        <v>1.68</v>
+      </c>
+      <c r="G27">
+        <v>39.35</v>
+      </c>
+      <c r="H27">
+        <f t="shared" si="4"/>
+        <v>2</v>
+      </c>
+      <c r="I27">
+        <f t="shared" si="6"/>
+        <v>2.7545000000000002</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -1212,4 +1465,677 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{442522CB-9026-483E-9FA1-CFE3429FB421}">
+  <dimension ref="A1:N26"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1">
+        <v>-3.52</v>
+      </c>
+      <c r="B1">
+        <v>-3.62</v>
+      </c>
+      <c r="C1">
+        <v>-3.42</v>
+      </c>
+      <c r="D1">
+        <v>0.12109499999999999</v>
+      </c>
+      <c r="E1">
+        <v>5.8891199999999998E-2</v>
+      </c>
+      <c r="F1">
+        <v>0</v>
+      </c>
+      <c r="I1">
+        <f t="shared" ref="I1:I16" si="0">A1+2.91</f>
+        <v>-0.60999999999999988</v>
+      </c>
+      <c r="J1">
+        <f t="shared" ref="J1:J16" si="1">B1+2.91</f>
+        <v>-0.71</v>
+      </c>
+      <c r="K1">
+        <f t="shared" ref="K1:K16" si="2">C1+2.91</f>
+        <v>-0.50999999999999979</v>
+      </c>
+      <c r="L1">
+        <v>31.160599999999999</v>
+      </c>
+      <c r="M1">
+        <v>5.2676699999999999</v>
+      </c>
+      <c r="N1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>-3.32</v>
+      </c>
+      <c r="B2">
+        <v>-3.42</v>
+      </c>
+      <c r="C2">
+        <v>-3.22</v>
+      </c>
+      <c r="D2">
+        <v>0.131217</v>
+      </c>
+      <c r="E2">
+        <v>4.7849099999999999E-2</v>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+      <c r="I2">
+        <f t="shared" si="0"/>
+        <v>-0.4099999999999997</v>
+      </c>
+      <c r="J2">
+        <f t="shared" si="1"/>
+        <v>-0.50999999999999979</v>
+      </c>
+      <c r="K2">
+        <f t="shared" si="2"/>
+        <v>-0.31000000000000005</v>
+      </c>
+      <c r="L2">
+        <v>28.376899999999999</v>
+      </c>
+      <c r="M2">
+        <v>4.3683100000000001</v>
+      </c>
+      <c r="N2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>-3.12</v>
+      </c>
+      <c r="B3">
+        <v>-3.22</v>
+      </c>
+      <c r="C3">
+        <v>-3.02</v>
+      </c>
+      <c r="D3">
+        <v>0.160663</v>
+      </c>
+      <c r="E3">
+        <v>4.4168399999999997E-2</v>
+      </c>
+      <c r="F3">
+        <v>0</v>
+      </c>
+      <c r="I3">
+        <f t="shared" si="0"/>
+        <v>-0.20999999999999996</v>
+      </c>
+      <c r="J3">
+        <f t="shared" si="1"/>
+        <v>-0.31000000000000005</v>
+      </c>
+      <c r="K3">
+        <f t="shared" si="2"/>
+        <v>-0.10999999999999988</v>
+      </c>
+      <c r="L3">
+        <v>27.7516</v>
+      </c>
+      <c r="M3">
+        <v>3.9400400000000002</v>
+      </c>
+      <c r="N3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>-2.92</v>
+      </c>
+      <c r="B4">
+        <v>-3.02</v>
+      </c>
+      <c r="C4">
+        <v>-2.82</v>
+      </c>
+      <c r="D4">
+        <v>0.177594</v>
+      </c>
+      <c r="E4">
+        <v>4.0487700000000001E-2</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="I4">
+        <f t="shared" si="0"/>
+        <v>-9.9999999999997868E-3</v>
+      </c>
+      <c r="J4">
+        <f t="shared" si="1"/>
+        <v>-0.10999999999999988</v>
+      </c>
+      <c r="K4">
+        <f t="shared" si="2"/>
+        <v>9.0000000000000302E-2</v>
+      </c>
+      <c r="L4">
+        <v>26.6296</v>
+      </c>
+      <c r="M4">
+        <v>3.5974300000000001</v>
+      </c>
+      <c r="N4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>-2.72</v>
+      </c>
+      <c r="B5">
+        <v>-2.82</v>
+      </c>
+      <c r="C5">
+        <v>-2.62</v>
+      </c>
+      <c r="D5">
+        <v>0.22728300000000001</v>
+      </c>
+      <c r="E5">
+        <v>3.5886800000000003E-2</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+      <c r="I5">
+        <f t="shared" si="0"/>
+        <v>0.18999999999999995</v>
+      </c>
+      <c r="J5">
+        <f t="shared" si="1"/>
+        <v>9.0000000000000302E-2</v>
+      </c>
+      <c r="K5">
+        <f t="shared" si="2"/>
+        <v>0.29000000000000004</v>
+      </c>
+      <c r="L5">
+        <v>28.7623</v>
+      </c>
+      <c r="M5">
+        <v>3.2119900000000001</v>
+      </c>
+      <c r="N5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>-2.52</v>
+      </c>
+      <c r="B6">
+        <v>-2.62</v>
+      </c>
+      <c r="C6">
+        <v>-2.42</v>
+      </c>
+      <c r="D6">
+        <v>0.27126800000000001</v>
+      </c>
+      <c r="E6">
+        <v>3.1285899999999998E-2</v>
+      </c>
+      <c r="F6">
+        <v>0</v>
+      </c>
+      <c r="I6">
+        <f t="shared" si="0"/>
+        <v>0.39000000000000012</v>
+      </c>
+      <c r="J6">
+        <f t="shared" si="1"/>
+        <v>0.29000000000000004</v>
+      </c>
+      <c r="K6">
+        <f t="shared" si="2"/>
+        <v>0.49000000000000021</v>
+      </c>
+      <c r="L6">
+        <v>30.886500000000002</v>
+      </c>
+      <c r="M6">
+        <v>2.7837299999999998</v>
+      </c>
+      <c r="N6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>-2.3199999999999998</v>
+      </c>
+      <c r="B7">
+        <v>-2.42</v>
+      </c>
+      <c r="C7">
+        <v>-2.2200000000000002</v>
+      </c>
+      <c r="D7">
+        <v>0.30255300000000002</v>
+      </c>
+      <c r="E7">
+        <v>2.3924500000000001E-2</v>
+      </c>
+      <c r="F7">
+        <v>0</v>
+      </c>
+      <c r="I7">
+        <f t="shared" si="0"/>
+        <v>0.5900000000000003</v>
+      </c>
+      <c r="J7">
+        <f t="shared" si="1"/>
+        <v>0.49000000000000021</v>
+      </c>
+      <c r="K7">
+        <f t="shared" si="2"/>
+        <v>0.69</v>
+      </c>
+      <c r="L7">
+        <v>32</v>
+      </c>
+      <c r="M7">
+        <v>2.14133</v>
+      </c>
+      <c r="N7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>-2.12</v>
+      </c>
+      <c r="B8">
+        <v>-2.2200000000000002</v>
+      </c>
+      <c r="C8">
+        <v>-2.02</v>
+      </c>
+      <c r="D8">
+        <v>0.34662999999999999</v>
+      </c>
+      <c r="E8">
+        <v>2.1163999999999999E-2</v>
+      </c>
+      <c r="F8">
+        <v>0</v>
+      </c>
+      <c r="I8">
+        <f t="shared" si="0"/>
+        <v>0.79</v>
+      </c>
+      <c r="J8">
+        <f t="shared" si="1"/>
+        <v>0.69</v>
+      </c>
+      <c r="K8">
+        <f t="shared" si="2"/>
+        <v>0.89000000000000012</v>
+      </c>
+      <c r="L8">
+        <v>34.646700000000003</v>
+      </c>
+      <c r="M8">
+        <v>1.8843700000000001</v>
+      </c>
+      <c r="N8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>-1.92</v>
+      </c>
+      <c r="B9">
+        <v>-2.02</v>
+      </c>
+      <c r="C9">
+        <v>-1.82</v>
+      </c>
+      <c r="D9">
+        <v>0.36033999999999999</v>
+      </c>
+      <c r="E9">
+        <v>1.74833E-2</v>
+      </c>
+      <c r="F9">
+        <v>0</v>
+      </c>
+      <c r="I9">
+        <f t="shared" si="0"/>
+        <v>0.99000000000000021</v>
+      </c>
+      <c r="J9">
+        <f t="shared" si="1"/>
+        <v>0.89000000000000012</v>
+      </c>
+      <c r="K9">
+        <f t="shared" si="2"/>
+        <v>1.0900000000000001</v>
+      </c>
+      <c r="L9">
+        <v>34.9893</v>
+      </c>
+      <c r="M9">
+        <v>1.54176</v>
+      </c>
+      <c r="N9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>-1.72</v>
+      </c>
+      <c r="B10">
+        <v>-1.82</v>
+      </c>
+      <c r="C10">
+        <v>-1.62</v>
+      </c>
+      <c r="D10">
+        <v>0.37892799999999999</v>
+      </c>
+      <c r="E10">
+        <v>1.84035E-2</v>
+      </c>
+      <c r="F10">
+        <v>0</v>
+      </c>
+      <c r="I10">
+        <f t="shared" si="0"/>
+        <v>1.1900000000000002</v>
+      </c>
+      <c r="J10">
+        <f t="shared" si="1"/>
+        <v>1.0900000000000001</v>
+      </c>
+      <c r="K10">
+        <f t="shared" si="2"/>
+        <v>1.29</v>
+      </c>
+      <c r="L10">
+        <v>36</v>
+      </c>
+      <c r="M10">
+        <v>1.54176</v>
+      </c>
+      <c r="N10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>-1.52</v>
+      </c>
+      <c r="B11">
+        <v>-1.62</v>
+      </c>
+      <c r="C11">
+        <v>-1.42</v>
+      </c>
+      <c r="D11">
+        <v>0.37616699999999997</v>
+      </c>
+      <c r="E11">
+        <v>2.2084199999999998E-2</v>
+      </c>
+      <c r="F11">
+        <v>0</v>
+      </c>
+      <c r="I11">
+        <f t="shared" si="0"/>
+        <v>1.3900000000000001</v>
+      </c>
+      <c r="J11">
+        <f t="shared" si="1"/>
+        <v>1.29</v>
+      </c>
+      <c r="K11">
+        <f t="shared" si="2"/>
+        <v>1.4900000000000002</v>
+      </c>
+      <c r="L11">
+        <v>35.5032</v>
+      </c>
+      <c r="M11">
+        <v>1.84154</v>
+      </c>
+      <c r="N11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>-1.32</v>
+      </c>
+      <c r="B12">
+        <v>-1.42</v>
+      </c>
+      <c r="C12">
+        <v>-1.22</v>
+      </c>
+      <c r="D12">
+        <v>0.350495</v>
+      </c>
+      <c r="E12">
+        <v>1.74833E-2</v>
+      </c>
+      <c r="F12">
+        <v>0</v>
+      </c>
+      <c r="I12">
+        <f t="shared" si="0"/>
+        <v>1.59</v>
+      </c>
+      <c r="J12">
+        <f t="shared" si="1"/>
+        <v>1.4900000000000002</v>
+      </c>
+      <c r="K12">
+        <f t="shared" si="2"/>
+        <v>1.6900000000000002</v>
+      </c>
+      <c r="L12">
+        <v>33.113500000000002</v>
+      </c>
+      <c r="M12">
+        <v>1.54176</v>
+      </c>
+      <c r="N12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>-1.1200000000000001</v>
+      </c>
+      <c r="B13">
+        <v>-1.22</v>
+      </c>
+      <c r="C13">
+        <v>-1.02</v>
+      </c>
+      <c r="D13">
+        <v>0.30071300000000001</v>
+      </c>
+      <c r="E13">
+        <v>1.38026E-2</v>
+      </c>
+      <c r="F13">
+        <v>0</v>
+      </c>
+      <c r="I13">
+        <f t="shared" si="0"/>
+        <v>1.79</v>
+      </c>
+      <c r="J13">
+        <f t="shared" si="1"/>
+        <v>1.6900000000000002</v>
+      </c>
+      <c r="K13">
+        <f t="shared" si="2"/>
+        <v>1.8900000000000001</v>
+      </c>
+      <c r="L13">
+        <v>28.8565</v>
+      </c>
+      <c r="M13">
+        <v>1.1991400000000001</v>
+      </c>
+      <c r="N13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>-0.92</v>
+      </c>
+      <c r="B14">
+        <v>-1.02</v>
+      </c>
+      <c r="C14">
+        <v>-0.82</v>
+      </c>
+      <c r="D14">
+        <v>0.25323200000000001</v>
+      </c>
+      <c r="E14">
+        <v>1.6563100000000001E-2</v>
+      </c>
+      <c r="F14">
+        <v>0</v>
+      </c>
+      <c r="I14">
+        <f t="shared" si="0"/>
+        <v>1.9900000000000002</v>
+      </c>
+      <c r="J14">
+        <f t="shared" si="1"/>
+        <v>1.8900000000000001</v>
+      </c>
+      <c r="K14">
+        <f t="shared" si="2"/>
+        <v>2.0900000000000003</v>
+      </c>
+      <c r="L14">
+        <v>24.907900000000001</v>
+      </c>
+      <c r="M14">
+        <v>1.4560999999999999</v>
+      </c>
+      <c r="N14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>-0.72</v>
+      </c>
+      <c r="B15">
+        <v>-0.82</v>
+      </c>
+      <c r="C15">
+        <v>-0.62</v>
+      </c>
+      <c r="D15">
+        <v>0.18900400000000001</v>
+      </c>
+      <c r="E15">
+        <v>1.38026E-2</v>
+      </c>
+      <c r="F15">
+        <v>0</v>
+      </c>
+      <c r="I15">
+        <f t="shared" si="0"/>
+        <v>2.1900000000000004</v>
+      </c>
+      <c r="J15">
+        <f t="shared" si="1"/>
+        <v>2.0900000000000003</v>
+      </c>
+      <c r="K15">
+        <f t="shared" si="2"/>
+        <v>2.29</v>
+      </c>
+      <c r="L15">
+        <v>19.357600000000001</v>
+      </c>
+      <c r="M15">
+        <v>1.1520300000000001</v>
+      </c>
+      <c r="N15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>-0.52</v>
+      </c>
+      <c r="B16">
+        <v>-0.62</v>
+      </c>
+      <c r="C16">
+        <v>-0.42</v>
+      </c>
+      <c r="D16">
+        <v>0.17244100000000001</v>
+      </c>
+      <c r="E16">
+        <v>2.9445599999999999E-2</v>
+      </c>
+      <c r="F16">
+        <v>0</v>
+      </c>
+      <c r="I16">
+        <f t="shared" si="0"/>
+        <v>2.39</v>
+      </c>
+      <c r="J16">
+        <f t="shared" si="1"/>
+        <v>2.29</v>
+      </c>
+      <c r="K16">
+        <f t="shared" si="2"/>
+        <v>2.4900000000000002</v>
+      </c>
+      <c r="L16">
+        <v>18.1328</v>
+      </c>
+      <c r="M16">
+        <v>2.6552500000000001</v>
+      </c>
+      <c r="N16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>11</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>